<commit_message>
Remplace le document Word par une feuille dediee dans le classeur Excel
Ajoute la feuille "Connexion GitHub" (colonne Commande isolee en police
monospace, une commande par ligne) pour un copier-coller direct - retire
le .docx, redondant et moins pratique pour cet usage.
</commit_message>
<xml_diff>
--- a/docs/TABLEAU_DE_BORD_EXPLOITATION.xlsx
+++ b/docs/TABLEAU_DE_BORD_EXPLOITATION.xlsx
@@ -3,17 +3,18 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="Demarrage rapide" sheetId="1" r:id="rId1"/>
-    <sheet name="Vocabulaire operateur" sheetId="2" r:id="rId2"/>
-    <sheet name="Correspondance Control-M" sheetId="3" r:id="rId3"/>
-    <sheet name="Bascule et exploitation" sheetId="4" r:id="rId4"/>
-    <sheet name="Demos resilience" sheetId="5" r:id="rId5"/>
+    <sheet name="Connexion GitHub" sheetId="2" r:id="rId2"/>
+    <sheet name="Vocabulaire operateur" sheetId="3" r:id="rId3"/>
+    <sheet name="Correspondance Control-M" sheetId="4" r:id="rId4"/>
+    <sheet name="Bascule et exploitation" sheetId="5" r:id="rId5"/>
+    <sheet name="Demos resilience" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
@@ -24,8 +25,18 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1F4E78"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Consolas"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -35,6 +46,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E6F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -51,11 +74,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -132,58 +164,70 @@
     <row r="6" ht="18">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">5. Premier lancement (VM1 d'abord)</t>
+          <t xml:space="preserve">5. Recuperer le projet</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">cd wazuh_factory_3 &amp;&amp; chmod +x orchestrator.sh jobs/*.sh &amp;&amp; ./orchestrator.sh -- laissez tourner jusqu'au bout (fail-fast : s'arrete proprement au premier probleme reel, avec le message exact).</t>
+          <t xml:space="preserve">Voir la feuille 'Connexion GitHub' - toutes les commandes de telechargement, prete a copier-coller.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">6. Premier lancement (VM2 ensuite)</t>
+          <t xml:space="preserve">6. Premier lancement (VM1 d'abord)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Copiez le meme dossier sur VM2, ROLE=AGENT_HOST dans vars.conf (deja pre-rempli), puis ./orchestrator.sh - VM2 va chercher automatiquement le certificat de la CA sur VM1 (SSH).</t>
+          <t xml:space="preserve">cd WEF &amp;&amp; chmod +x orchestrator.sh jobs/*.sh &amp;&amp; ./orchestrator.sh -- laissez tourner jusqu'au bout (fail-fast : s'arrete proprement au premier probleme reel, avec le message exact).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7. Ou trouver les identifiants generes</t>
+          <t xml:space="preserve">7. Premier lancement (VM2 ensuite)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aucun mot de passe n'est ecrit en dur nulle part. Une fois l'installation terminee : sourcez operator_profile.sh puis tapez 'escreds' (affiche Kibana/Elasticsearch) - pour Wazuh Dashboard, voir secrets/wazuh_indexer_admin_password.txt.</t>
+          <t xml:space="preserve">Copiez le meme dossier sur VM2, ROLE=AGENT_HOST dans vars.conf (deja pre-rempli), puis ./orchestrator.sh - VM2 va chercher automatiquement le certificat de la CA sur VM1 (SSH).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">8. Tableau de bord visuel live (recommande pour la demo)</t>
+          <t xml:space="preserve">8. Ou trouver les identifiants generes</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">./installer_service_tableau_de_bord.sh puis ouvrez http://&lt;IP_VM1&gt;:&lt;PORT&gt; - vue graphique type 'Monitoring Domain' Control-M, mise a jour en direct, aucune action possible depuis cette page (lecture seule).</t>
+          <t xml:space="preserve">Aucun mot de passe n'est ecrit en dur nulle part. Une fois l'installation terminee : sourcez operator_profile.sh puis tapez 'escreds' (affiche Kibana/Elasticsearch) - pour Wazuh Dashboard, voir secrets/wazuh_indexer_admin_password.txt.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">9. Pour la suite</t>
+          <t xml:space="preserve">9. Tableau de bord visuel live (recommande pour la demo)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./installer_service_tableau_de_bord.sh puis ouvrez http://&lt;IP_VM1&gt;:&lt;PORT&gt; - vue graphique type 'Monitoring Domain' Control-M, mise a jour en direct, aucune action possible depuis cette page (lecture seule).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10. Pour la suite</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t xml:space="preserve">Voir feuille 'Vocabulaire operateur' (commandes courtes du quotidien) et 'Correspondance Control-M' (equivalences avec les actions que vous connaissez deja).</t>
         </is>
@@ -194,6 +238,460 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="2" width="68" customWidth="1"/>
+    <col min="3" max="3" width="55" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Etape</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Commande (copier-coller)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Remarque</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32">
+      <c r="A2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">⚠ Depot public (https://github.com/ykeupssi123-ship-it/WEF) : aucun compte GitHub n'est necessaire pour le telecharger. Un compte n'est requis que pour la section C (optionnelle).</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20">
+      <c r="A3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A. Cas normal - cloner directement sur les VM Linux (VM1 et VM2)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Verifier que git est present</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">git --version</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Si 'command not found', passer a l'etape 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. Installer git si absent</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">sudo dnf install -y git</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Reverifier</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">git --version</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ne pas continuer si erreur</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Se placer dans le dossier de travail</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">cd ~</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5. Cloner le depot</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">git clone https://github.com/ykeupssi123-ship-it/WEF.git</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Depot public, aucune authentification requise</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6. Entrer dans le dossier</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">cd WEF</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7. Verifier l'etat du clone</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">git status</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doit afficher : On branch main / nothing to commit, working tree clean</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8. Compter les scripts recuperes</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">find . -name "*.sh" | wc -l</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doit etre proche de 260 - sinon clone incomplet, refaire l'etape 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9. Rendre les scripts executables</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">chmod +x orchestrator.sh jobs/*.sh</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatoire - Git ne preserve pas les droits Unix depuis un clone HTTPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10. Lancer (VM1)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">./orchestrator.sh</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ROLE=ELK_HOST deja par defaut dans vars.conf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10bis. Lancer (VM2)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">./orchestrator.sh</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Avant : changer ROLE=AGENT_HOST dans vars.conf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20">
+      <c r="A15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B. Alternative sans git (si son installation est refusee/impossible)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11. Telecharger l'archive ZIP</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">curl -L -o WEF.zip https://github.com/ykeupssi123-ship-it/WEF/archive/refs/heads/main.zip</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12. Extraire</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">unzip WEF.zip</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13. Entrer dans le dossier</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">cd WEF-main</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14. Rendre executable</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">chmod +x orchestrator.sh jobs/*.sh</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20">
+      <c r="A20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">C. Optionnel - creer un compte GitHub personnel (fork, contribution)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15. Creer un compte</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">https://github.com/signup</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dans un navigateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16. Configurer l'identite Git (nom)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">git config --global user.name "Prenom Nom"</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Une seule fois par machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17. Configurer l'identite Git (email)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">git config --global user.email "email@exemple.com"</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Une seule fois par machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18. Forker le depot</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">https://github.com/ykeupssi123-ship-it/WEF</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bouton 'Fork' en haut a droite - cree une copie personnelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19. Cloner sa propre copie</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">git clone https://github.com/SON-COMPTE/WEF.git</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Remplacer SON-COMPTE par le nom d'utilisateur reel</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20. Generer un token d'acces (pour git push)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">https://github.com/settings/tokens</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Utilise comme mot de passe au premier git push - jamais le mot de passe du compte</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -375,7 +873,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -718,7 +1216,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -900,7 +1398,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>

</xml_diff>

<commit_message>
Etoffe le classeur d'exploitation : deploiement VM2/Windows + arborescence
- Feuille "Deploiement VM2 (agent Linux)" : prerequis SSH VM2->VM1 (cle ou
  mot de passe+sshpass) pour que DIST_001 recupere la CA sans bloquer,
  puis sequence de deploiement complete.
- Feuille "Deploiement agent Windows" : recuperation du kit, depot manuel
  du certificat CA (pscp), lancement, et configuration DNS optionnelle de
  l'interface VMnet8 pour resoudre les noms internes depuis le poste.
- Feuille "Arborescence exploitation" : vue curatee par domaine (bascule,
  sante/auto-guerison, demos resilience, verifications) avec explication
  en langage clair de ce que sert chaque job, pas seulement son ID.
- Feuille "Reference complete jobs RUN" : les 78 jobs RUN du projet,
  annexe exhaustive.
</commit_message>
<xml_diff>
--- a/docs/TABLEAU_DE_BORD_EXPLOITATION.xlsx
+++ b/docs/TABLEAU_DE_BORD_EXPLOITATION.xlsx
@@ -4,10 +4,14 @@
   <sheets>
     <sheet name="Demarrage rapide" sheetId="1" r:id="rId1"/>
     <sheet name="Connexion GitHub" sheetId="2" r:id="rId2"/>
-    <sheet name="Vocabulaire operateur" sheetId="3" r:id="rId3"/>
-    <sheet name="Correspondance Control-M" sheetId="4" r:id="rId4"/>
-    <sheet name="Bascule et exploitation" sheetId="5" r:id="rId5"/>
-    <sheet name="Demos resilience" sheetId="6" r:id="rId6"/>
+    <sheet name="Deploiement VM2 (agent Linux)" sheetId="3" r:id="rId3"/>
+    <sheet name="Deploiement agent Windows" sheetId="4" r:id="rId4"/>
+    <sheet name="Arborescence exploitation" sheetId="5" r:id="rId5"/>
+    <sheet name="Vocabulaire operateur" sheetId="6" r:id="rId6"/>
+    <sheet name="Correspondance Control-M" sheetId="7" r:id="rId7"/>
+    <sheet name="Bascule et exploitation" sheetId="8" r:id="rId8"/>
+    <sheet name="Demos resilience" sheetId="9" r:id="rId9"/>
+    <sheet name="Reference complete jobs RUN" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -237,6 +241,1757 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="65" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ID Job</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Role machine</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Commande</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_027</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Pression : Polling local actif de l'API</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_027 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_028</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fiche [USB 2.3] : Pipeline d'ingestion brute JSON</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_028 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_029</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fiche [USB 3.0] : Pipeline d'ingestion Syslog RFC5424</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_029 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_030</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fiche [RJ45 SEC] : Pipeline decodage Common Event Format</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_030 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_031</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fiche [SERIE / TEXT] : Pipeline de traitement de fichiers plats CSV</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_031 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_032</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fiche [SATELLITE] : Pipeline de decodage des structures XML Windows</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_032 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_033</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adaptateur Horloge : Normalisation universelle temporelle</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_033 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_034</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Filtre Securite : Suppresseur universel de donnees sensibles</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_034 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_035</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Filtre Debit : Disjoncteur automatique de logs parasites</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_035 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_036</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Raccordement : Validation fonctionnelle des fiches</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_036 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_037</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle de Vie : Definition des regles de purge et de rollover</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_037 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_038</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chassis Logique : Parametres d'indexation globaux (1 Shard)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_038 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_039</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chassis Logique : Schema de reception dynamic keyword</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_039 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_040</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assemblage Prise : Creation du gabarit d'interception log-*</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_040 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_041</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Disjoncteur Cluster : Verrouillage des index hors gabarit</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_041 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_043</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Rigueur : Validation du verrouillage memoire RAM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_043 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_044</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Charge : Verification reelle des descripteurs</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_044 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_045</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Isolation : Rejet des acces reseau non chiffres</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_045 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_046</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Epreuve de Pression : Simulation de charge d'ingestion</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_046 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_049</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Masse : Evaluation de la reserve physique utile</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_049 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_050</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prise Universelle : Armement du compte d'ingestion mutualise</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_050 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_050B</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prise Universelle (alternative) : armement du compte d'ingestion par mot de passe</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_050B "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_051</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simulation Sinistre : Arret brutal par destruction du PID</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_051 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_052</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verification Relance : Redemarrage apres sinistre</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_052 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_053</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Sante : Reponse de l'API post-destruction</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_053 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_054</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Memoire : Persistance des ports logiques injectes</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_054 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_055</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Epreuve Volatile : Redemarrage complet a froid du demon de l'OS</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_055 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_056</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Epreuve Volatile : Polling de reactivite post-purge RAM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_056 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_057</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Epreuve Volatile : Maintien de l'isolation du pare-feu</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_057 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_058</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Epreuve Volatile : Persistance des identifiants maitres</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_058 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_061</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vanne Maitresse : Emission de la condition globale</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_061 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS_021</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Filtre Ethique : Anonymisation des cartes bancaires (PCI-DSS)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh LS_021 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS_022</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Filtre Ethique : Suppression des mots de passe en clair</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh LS_022 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS_023</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enrichment : Activation du module GeoIP pour tracabilite</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh LS_023 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS_027</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Pression : Analyse du fichier de demarrage</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh LS_027 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS_028</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Raccordement : Polling de l'API locale (9600)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh LS_028 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS_029</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crash Test : Simulation d'absence totale du moteur de stockage local</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh LS_029 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS_030</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Epreuve de Charge : Agression de la prise en mode isole</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh LS_030 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS_031</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Derivation : Verification du stockage temporaire (Persistent Queues)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh LS_031 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS_032</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Disjoncteur : Injection d'un log corrompu (Crash-test structure)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh LS_032 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS_033</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retablissement : Reouverture des vannes de communication locales</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh LS_033 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS_035_PREP</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vanne Maitresse : Emission du signal d'independance absolue</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh LS_035_PREP "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB_019</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Pression : Verification de l'ecoute du port 5601</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh KB_019 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB_020</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Lucidite : Polling de l'API de statut interne</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh KB_020 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB_021</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crash Test : Blocage artificiel du port local de la base de donnees</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh KB_021 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB_022</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Epreuve de Solidite : Tentative d'acces a l'interface pendant l'isolement</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh KB_022 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB_025</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prise de Sortie : Extraction instantanee des structures de rendu</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh KB_025 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="18">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB_026</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prise d'Entree : Injection a chaud de configurations industrielles</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh KB_026 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB_029</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vanne Maitresse : Emission du signal de disponibilite du Hub</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh KB_029 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FB_015</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AGENT_HOST</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crash Test : Simulation d'extinction du monde exterieur</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh FB_015 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FB_016</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AGENT_HOST</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Epreuve de Charge : Agression des entrees en mode isole</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh FB_016 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FB_017</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AGENT_HOST</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Memoire : Validation du pointeur de lecture local</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh FB_017 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FB_018</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AGENT_HOST</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Derivation : Verification du maintien de la structure</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh FB_018 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MB_015</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AGENT_HOST</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crash Test : Simulation de disparition de l'infrastructure reseau</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh MB_015 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MB_016</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AGENT_HOST</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Epreuve de Charge : Faux pics d'activite systeme en isolation</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh MB_016 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MB_017</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AGENT_HOST</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Retention : Verification de la non-perte des paquets de telemetrie</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh MB_017 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_014A_INDXR_ADMINPW</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Authentification : Alignement du mot de passe admin reel sur vars.conf</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_014A_INDXR_ADMINPW "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="18">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_017E_AUTHAPPLY</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Authentification (optionnel) : application du mode choisi</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_017E_AUTHAPPLY "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="18">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_018_NET</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crash Test Reseau : Rupture artificielle des flux reseau sortants</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_018_NET "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="18">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_019_FLOOD</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Epreuve de Charge : Simulation d'un deluge massif d'evenements</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_019_FLOOD "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="18">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_020_VERIFY</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Retention : Verification de la bonne inscription locale</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_020_VERIFY "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="18">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_027</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simulation Sinistre : Arret brutal du manager par destruction de PID</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_027 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="18">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_028</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verification Relance : Redemarrage et controle post-sinistre</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_028 "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="18">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_035_MODE_CONVERGENT</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vanne Un-Clic : bascule EXCLUSIVE des alertes vers Elasticsearch/Kibana</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_035_MODE_CONVERGENT "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="18">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_037_CONVERGENT_TEST</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Preuve Reelle Convergence : injecte une alerte reelle et verifie sa presence dans Elasticsearch</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_037_CONVERGENT_TEST "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="18">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_038_KIBANA_VERIFY</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Presence : Verification de la vivacite de l'index usine</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_038_KIBANA_VERIFY "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="18">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_039_MODE_SOUVERAIN</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vanne Un-Clic Reversible : bascule EXCLUSIVE des alertes vers wazuh-indexer</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_039_MODE_SOUVERAIN "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="18">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_040_KIBANA_SILENT</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controle Etancheite : verifie l'exclusivite reelle de la destination</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_040_KIBANA_SILENT "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="18">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_041_ALERT_CANARY</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exploitation continue : test d'alerte synthetique quotidien</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_041_ALERT_CANARY "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="18">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_042_INDEXER_UNLOCK</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exploitation continue : leve les verrous lecture-seule (flood-stage)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_042_INDEXER_UNLOCK "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="18">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_043_DASHBOARD_FIELDS_REFRESH</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exploitation continue : purge le cache de champs perime du Dashboard</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_043_DASHBOARD_FIELDS_REFRESH "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="18">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAZ_044_VD_SAFE_RETRY</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exploitation continue : relance surveillee du Vulnerability Detector</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_044_VD_SAFE_RETRY "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="18">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INFRA_004_HEALTH_GUARDIAN</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALL</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exploitation continue : controle de sante toutes les 5 min</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh INFRA_004_HEALTH_GUARDIAN "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="18">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INFRA_005_DISK_HYGIENE</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALL</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exploitation continue : entretien disque hebdomadaire permanent</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh INFRA_005_DISK_HYGIENE "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="18">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DNS_004_START</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DNS interne : demarrage + verification reelle de la resolution des FQDN</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh DNS_004_START "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="18">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_062_SNAPSHOTS3REPO</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sauvegarde (optionnelle) : enregistrement du depot de snapshots S3 OVH</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_062_SNAPSHOTS3REPO "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="18">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES_063_SNAPSHOTPOLICY</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELK_HOST</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sauvegarde (optionnelle) : politique de cycle de vie des snapshots (SLM)</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_063_SNAPSHOTPOLICY "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="18">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAG_006</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AGENT_HOST</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verification enregistrement et rapport final (agent Wazuh Linux)</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAG_006 "raison"</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
@@ -694,6 +2449,1045 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="2" width="68" customWidth="1"/>
+    <col min="3" max="3" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Etape</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Commande</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Remarque</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32">
+      <c r="A2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">⚠ DIST_001 recupere AUTOMATIQUEMENT le certificat de la CA d'usine depuis VM1 des le premier lancement de l'orchestrateur sur VM2 - ce n'est jamais une commande a jouer a la main. Mais il lui faut un acces SSH VM2 -&gt; VM1 deja pret : choisissez UNE des deux options ci-dessous AVANT de lancer ./orchestrator.sh.</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20">
+      <c r="A3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Prerequis - Option recommandee : cle SSH (a executer sur VM2)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Generer une cle SSH (si absente)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">ssh-keygen -t ed25519 -N "" -f ~/.ssh/id_ed25519</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Une seule fois par machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. Copier la cle publique sur VM1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">ssh-copy-id root@192.168.50.128</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Demande le mot de passe root de VM1 - une seule fois</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Verifier la connexion sans mot de passe</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">ssh root@192.168.50.128 "echo OK"</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doit repondre OK sans rien demander - sinon ne pas continuer</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Indiquer le chemin de la cle</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">FACTORY_SSH_KEY="/root/.ssh/id_ed25519"</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ligne a editer dans vars.conf sur VM2 (remplace la valeur vide par defaut)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20">
+      <c r="A8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Prerequis - Option de secours : mot de passe SSH (VM2 uniquement, jamais sur VM1)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5. Installer sshpass</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">sudo dnf install -y sshpass</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Necessaire uniquement pour cette option</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6. Deposer le mot de passe root de VM1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">echo 'mot_de_passe_root_VM1' &gt; secrets/factory_ssh_password.txt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jamais dans vars.conf, jamais sur VM1 - uniquement ce fichier, sur VM2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7. Restreindre les droits du fichier</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">chmod 600 secrets/factory_ssh_password.txt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20">
+      <c r="A12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Deploiement (identique a VM1, avec ROLE=AGENT_HOST)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8. Cloner le depot</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">git clone https://github.com/ykeupssi123-ship-it/WEF.git</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voir feuille 'Connexion GitHub' pour le detail complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9. Entrer dans le dossier</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">cd WEF</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10. Regler le role de cette machine</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">ROLE="AGENT_HOST"</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ligne a editer dans vars.conf (remplace ROLE=ELK_HOST)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11. Verifier les composants actives</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">AGENT_COMPONENTS="FILEBEAT,METRICBEAT,WAZUH_AGENT,HOSTNAME_RENAME"</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valeur par defaut - les 3 agents tournent sur la meme machine VM2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12. Rendre les scripts executables</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">chmod +x orchestrator.sh jobs/*.sh</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13. Lancer</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">./orchestrator.sh</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIST_001 recupere la CA a ce moment - echoue proprement avec un message clair si l'etape 1-7 n'a pas ete faite</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="75" customWidth="1"/>
+    <col min="3" max="3" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Etape</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Commande</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Remarque</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32">
+      <c r="A2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">⚠ Toutes les commandes ci-dessous s'executent dans PowerShell EN ADMINISTRATEUR, sur la machine Windows a equiper (physique ou VM).</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20">
+      <c r="A3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Recuperer le projet (sans git - simple ZIP)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Telecharger l'archive</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Invoke-WebRequest -Uri https://github.com/ykeupssi123-ship-it/WEF/archive/refs/heads/main.zip -OutFile WEF.zip</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. Extraire</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Expand-Archive WEF.zip -DestinationPath .</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Entrer dans le dossier du kit Windows</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">cd WEF-main\jobs_windows</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20">
+      <c r="A7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">2. Recuperer le certificat de la CA d'usine (depuis VM1)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32">
+      <c r="A8" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">⚠ Aucun canal automatique depuis ce kit (contrairement a DIST_001 cote Linux) - obligatoire si FILEBEAT ou METRICBEAT reste active dans vars.ps1, sinon FBW_004/MBW_004 arretent le job avec un message clair plutot que d'improviser.</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Creer le dossier de destination</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">New-Item -ItemType Directory -Force -Path C:\ProgramData\wef-pki</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5. Recuperer le certificat depuis VM1 (pscp, PuTTY)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">pscp root@192.168.50.128:/etc/pki/factory/certs/factory_ca.crt C:\ProgramData\wef-pki\factory_ca.crt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Demande le mot de passe root de VM1 - pscp fourni par l'installation PuTTY</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20">
+      <c r="A11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3. Configurer cette machine</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6. Ouvrir vars.ps1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">notepad vars.ps1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Changer $AGENT_NAME (unique par machine) et $EnabledComponents si besoin</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20">
+      <c r="A13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">4. Lancer</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7. Autoriser l'execution de scripts (session en cours)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Set-ExecutionPolicy -Scope Process -ExecutionPolicy Bypass</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PowerShell doit etre ouvert EN ADMINISTRATEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8. Lancer l'orchestrateur</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">.\orchestrator_windows.ps1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Installe agent Wazuh + Filebeat + Metricbeat selon $EnabledComponents</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20">
+      <c r="A16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5. Optionnel - resoudre dashboard.wef.local / kibana.wef.local depuis ce poste</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32">
+      <c r="A17" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">⚠ Sans effet sur le fonctionnement des agents (ils utilisent l'IP directement, jamais un nom) - utile seulement pour ouvrir les tableaux de bord dans un navigateur avec un nom plutot qu'une adresse IP. Non teste dans cet environnement (pas de PowerShell disponible cote assistant) - a verifier une fois en reel.</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9. Identifier le nom exact de l'interface VMnet8</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Get-NetAdapter | Where-Object {$_.InterfaceDescription -like "*VMnet8*"}</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notez la colonne Name - le nom peut varier selon l'installation VMware</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10. Definir VM1 comme serveur DNS sur cette interface</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Set-DnsClientServerAddress -InterfaceAlias "VMware Network Adapter VMnet8" -ServerAddresses 192.168.50.128</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Remplacer le nom d'interface si different de l'etape precedente</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11. Vider le cache DNS local</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">ipconfig /flushdns</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12. Verifier la resolution</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Resolve-DnsName dashboard.wef.local</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doit renvoyer 192.168.50.128</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13. Revenir a la resolution DNS normale (si besoin)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Set-DnsClientServerAddress -InterfaceAlias "VMware Network Adapter VMnet8" -ResetServerAddresses</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annule l'etape 10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="2" width="85" customWidth="1"/>
+    <col min="3" max="3" width="45" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Domaine / Job</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">A quoi ca sert (en clair)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Commande</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32">
+      <c r="A2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">⚠ Vue curatee (l'essentiel du quotidien) - la liste complete des 78 jobs RUN du projet est dans la feuille 'Reference complete jobs RUN'.</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20">
+      <c r="A3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. BASCULE D'EXPLOITATION - le coeur du systeme, le geste le plus frequent</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WAZ_035_MODE_CONVERGENT</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Basculer la vue vers Kibana - pour explorer/analyser en profondeur avec les outils ELK classiques.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_035_MODE_CONVERGENT "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WAZ_039_MODE_SOUVERAIN</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Revenir a Wazuh Dashboard - l'etat normal de securite, celui qu'on laisse tourner par defaut.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_039_MODE_SOUVERAIN "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20">
+      <c r="A6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">2. SANTE ET AUTO-GUERISON - ce qui tourne tout seul, jamais a declencher a la main sauf urgence</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WAZ_041_ALERT_CANARY</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Preuve de vie quotidienne automatique (06h) - detecte un pipeline d'alertes mort en silence, avant qu'un humain ne s'en rende compte par hasard.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_041_ALERT_CANARY "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    INFRA_004_HEALTH_GUARDIAN</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Garde-fou toutes les 5 minutes - verifie services/DNS/certificat/disque, alerte au premier ecart.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh INFRA_004_HEALTH_GUARDIAN "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    INFRA_005_DISK_HYGIENE</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Nettoyage automatique chaque dimanche 03h - evite la panne par disque plein avant qu'elle n'arrive.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh INFRA_005_DISK_HYGIENE "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WAZ_042_INDEXER_UNLOCK</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Debloque l'ecriture si un episode de disque plein a laisse des verrous - a jouer si le Dashboard n'affiche plus rien de nouveau.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_042_INDEXER_UNLOCK "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WAZ_043_DASHBOARD_FIELDS_REFRESH</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Repare l'affichage si des panneaux montrent une erreur de champ (ex: apres un changement de mapping).</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_043_DASHBOARD_FIELDS_REFRESH "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WAZ_044_VD_SAFE_RETRY</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Relance le scanner de vulnerabilites en toute securite (verifie la place disque avant).</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_044_VD_SAFE_RETRY "raison"</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20">
+      <c r="A13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3. DEMONSTRATIONS DE RESILIENCE - pour montrer, devant un jury ou un client, que le systeme encaisse une panne</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ES_051 -&gt; ES_052 -&gt; ES_053</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Elasticsearch : on le tue brutalement (051), on prouve qu'il redemarre tout seul (052), on confirme qu'il repond de nouveau normalement (053).</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh ES_051 "raison"  (puis 052, puis 053)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WAZ_027 -&gt; WAZ_028</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Wazuh manager : meme scenario - arret brutal (027) puis preuve de reprise reelle (028), jamais un 'OK' suppose.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh WAZ_027 "raison"  (puis WAZ_028)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    KB_021 -&gt; KB_022</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Kibana : on l'isole artificiellement de sa base (021), on prouve que l'interface reste consultable en degrade (022).</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh KB_021 "raison"  (puis KB_022)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    LS_029 -&gt; LS_031 -&gt; LS_033</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Logstash : on simule l'absence totale de stockage (029), on prouve que rien n'est perdu (file d'attente locale, 031), on retablit et on confirme (033).</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh LS_029 "raison"  (puis 031, puis 033)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20">
+      <c r="A18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">4. VERIFICATIONS DE ROUTINE - moins spectaculaire, mais ce qui prouve qu'une etape a vraiment reussi</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ES_027 / KB_019-020 / LS_027-028</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Controles de sante ponctuels (API repond, port ecoute, pipeline demarre) - surtout utiles en diagnostic, rarement rejoues seuls en exploitation courante.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./forcer_job.sh &lt;ID&gt; "raison"</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="70" customWidth="1"/>
     <col min="3" max="3" width="55" customWidth="1"/>
@@ -873,7 +3667,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1216,7 +4010,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1398,7 +4192,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>

</xml_diff>

<commit_message>
Ajoute les prerequis systeme reels de VM2 avant tout lancement
Section 0 (feuille "Deploiement VM2") : IP statique via nmcli (interface,
passerelle et DNS verifies reellement sur VM1, meme reseau attendu),
test de joignabilite vers VM1, port SSH, et rappel qu'aucun controle
RAM/disque automatique n'existe pour AGENT_HOST (a l'inverse de VM1) -
a verifier a la main.
</commit_message>
<xml_diff>
--- a/docs/TABLEAU_DE_BORD_EXPLOITATION.xlsx
+++ b/docs/TABLEAU_DE_BORD_EXPLOITATION.xlsx
@@ -2474,7 +2474,7 @@
     <row r="2" ht="32">
       <c r="A2" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">⚠ DIST_001 recupere AUTOMATIQUEMENT le certificat de la CA d'usine depuis VM1 des le premier lancement de l'orchestrateur sur VM2 - ce n'est jamais une commande a jouer a la main. Mais il lui faut un acces SSH VM2 -&gt; VM1 deja pret : choisissez UNE des deux options ci-dessous AVANT de lancer ./orchestrator.sh.</t>
+          <t xml:space="preserve">⚠ Rien de ce qui suit dans la section 0 n'est fait par l'orchestrateur - ce sont des prerequis SYSTEME (reseau, ressources), verifies ici a la main une seule fois avant le premier lancement. Aucun controle RAM/disque automatique n'existe pour AGENT_HOST (contrairement a VM1, voir ES_B001_RAM_CHECK) - limite honnete, a verifier soi-meme.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="4">
@@ -2491,7 +2491,7 @@
     <row r="3" ht="20">
       <c r="A3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Prerequis - Option recommandee : cle SSH (a executer sur VM2)</t>
+          <t xml:space="preserve">0. Prerequis machine (rien n'est encore installe a ce stade)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="2">
@@ -2508,253 +2508,389 @@
     <row r="4" ht="18">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Generer une cle SSH (si absente)</t>
+          <t xml:space="preserve">0.1 Identifier le nom de l'interface reseau</t>
         </is>
       </c>
       <c r="B4" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">ssh-keygen -t ed25519 -N "" -f ~/.ssh/id_ed25519</t>
+          <t xml:space="preserve">nmcli device status</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Une seule fois par machine</t>
+          <t xml:space="preserve">Cherchez le type 'ethernet' - le nom (ens160, ens192, eth0...) peut differer de VM1 selon le clone/modele utilise</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. Copier la cle publique sur VM1</t>
+          <t xml:space="preserve">0.2 Fixer une IP statique (192.168.50.130)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">ssh-copy-id root@192.168.50.128</t>
+          <t xml:space="preserve">nmcli connection modify "ens160" ipv4.addresses 192.168.50.130/24 ipv4.gateway 192.168.50.2 ipv4.dns 8.8.8.8 ipv4.method manual</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demande le mot de passe root de VM1 - une seule fois</t>
+          <t xml:space="preserve">Remplacer "ens160" par le nom reel trouve a l'etape 0.1. Valeurs de passerelle/DNS verifiees reelles sur VM1 (meme reseau VMware attendu)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. Verifier la connexion sans mot de passe</t>
+          <t xml:space="preserve">0.3 Appliquer</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">ssh root@192.168.50.128 "echo OK"</t>
+          <t xml:space="preserve">nmcli connection up "ens160"</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doit repondre OK sans rien demander - sinon ne pas continuer</t>
+          <t xml:space="preserve">Meme nom qu'a l'etape 0.2 - une coupure bref de la session SSH en cours est normale si vous etiez deja connecte en DHCP</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. Indiquer le chemin de la cle</t>
+          <t xml:space="preserve">0.4 Verifier l'adresse appliquee</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">FACTORY_SSH_KEY="/root/.ssh/id_ed25519"</t>
+          <t xml:space="preserve">ip addr show</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ligne a editer dans vars.conf sur VM2 (remplace la valeur vide par defaut)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20">
-      <c r="A8" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Prerequis - Option de secours : mot de passe SSH (VM2 uniquement, jamais sur VM1)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Doit afficher inet 192.168.50.130/24 sur l'interface</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.5 Verifier que VM1 est joignable</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">ping -c 3 192.168.50.128</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doit repondre - sinon revoir le reseau virtuel (les 2 VM doivent etre sur le meme commutateur virtuel, ex: VMnet8) avant de continuer</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">5. Installer sshpass</t>
+          <t xml:space="preserve">0.6 Verifier le port SSH de VM1 ouvert</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">sudo dnf install -y sshpass</t>
+          <t xml:space="preserve">nc -zv 192.168.50.128 22</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Necessaire uniquement pour cette option</t>
+          <t xml:space="preserve">'succeeded' attendu - necessaire pour DIST_001 (section suivante) et pour cloner/administrer a distance</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">6. Deposer le mot de passe root de VM1</t>
+          <t xml:space="preserve">0.7 Verifier les ressources de CETTE machine</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">echo 'mot_de_passe_root_VM1' &gt; secrets/factory_ssh_password.txt</t>
+          <t xml:space="preserve">nproc &amp;&amp; free -h &amp;&amp; df -h /</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jamais dans vars.conf, jamais sur VM1 - uniquement ce fichier, sur VM2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7. Restreindre les droits du fichier</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">chmod 600 secrets/factory_ssh_password.txt</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20">
-      <c r="A12" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Deploiement (identique a VM1, avec ROLE=AGENT_HOST)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Minimum recommande : 2 vCPU / 4 Go RAM / 20 Go disque (jamais verifie automatiquement pour VM2, a l'inverse de VM1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20">
+      <c r="A11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Prerequis - Option recommandee : cle SSH (a executer sur VM2)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Generer une cle SSH (si absente)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">ssh-keygen -t ed25519 -N "" -f ~/.ssh/id_ed25519</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Une seule fois par machine</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">8. Cloner le depot</t>
+          <t xml:space="preserve">2. Copier la cle publique sur VM1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">git clone https://github.com/ykeupssi123-ship-it/WEF.git</t>
+          <t xml:space="preserve">ssh-copy-id root@192.168.50.128</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voir feuille 'Connexion GitHub' pour le detail complet</t>
+          <t xml:space="preserve">Demande le mot de passe root de VM1 - une seule fois</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">9. Entrer dans le dossier</t>
+          <t xml:space="preserve">3. Verifier la connexion sans mot de passe</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">cd WEF</t>
+          <t xml:space="preserve">ssh root@192.168.50.128 "echo OK"</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Doit repondre OK sans rien demander - sinon ne pas continuer</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">10. Regler le role de cette machine</t>
+          <t xml:space="preserve">4. Indiquer le chemin de la cle</t>
         </is>
       </c>
       <c r="B15" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">ROLE="AGENT_HOST"</t>
+          <t xml:space="preserve">FACTORY_SSH_KEY="/root/.ssh/id_ed25519"</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ligne a editer dans vars.conf (remplace ROLE=ELK_HOST)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11. Verifier les composants actives</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">AGENT_COMPONENTS="FILEBEAT,METRICBEAT,WAZUH_AGENT,HOSTNAME_RENAME"</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Valeur par defaut - les 3 agents tournent sur la meme machine VM2</t>
+          <t xml:space="preserve">Ligne a editer dans vars.conf sur VM2 (remplace la valeur vide par defaut)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20">
+      <c r="A16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Prerequis - Option de secours : mot de passe SSH (VM2 uniquement, jamais sur VM1)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="17" ht="18">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">12. Rendre les scripts executables</t>
+          <t xml:space="preserve">5. Installer sshpass</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">chmod +x orchestrator.sh jobs/*.sh</t>
+          <t xml:space="preserve">sudo dnf install -y sshpass</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Necessaire uniquement pour cette option</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t xml:space="preserve">6. Deposer le mot de passe root de VM1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">echo 'mot_de_passe_root_VM1' &gt; secrets/factory_ssh_password.txt</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jamais dans vars.conf, jamais sur VM1 - uniquement ce fichier, sur VM2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7. Restreindre les droits du fichier</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">chmod 600 secrets/factory_ssh_password.txt</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20">
+      <c r="A20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Deploiement (identique a VM1, avec ROLE=AGENT_HOST)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8. Cloner le depot</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">git clone https://github.com/ykeupssi123-ship-it/WEF.git</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voir feuille 'Connexion GitHub' pour le detail complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9. Entrer dans le dossier</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">cd WEF</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10. Regler le role de cette machine</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">ROLE="AGENT_HOST"</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ligne a editer dans vars.conf (remplace ROLE=ELK_HOST)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11. Verifier les composants actives</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">AGENT_COMPONENTS="FILEBEAT,METRICBEAT,WAZUH_AGENT,HOSTNAME_RENAME"</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valeur par defaut - les 3 agents tournent sur la meme machine VM2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12. Rendre les scripts executables</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">chmod +x orchestrator.sh jobs/*.sh</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18">
+      <c r="A26" t="inlineStr">
+        <is>
           <t xml:space="preserve">13. Lancer</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr" s="3">
+      <c r="B26" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">./orchestrator.sh</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t xml:space="preserve">DIST_001 recupere la CA a ce moment - echoue proprement avec un message clair si l'etape 1-7 n'a pas ete faite</t>
         </is>

</xml_diff>

<commit_message>
Corrige l'angle mort : aucun controle de ressources n'existait pour AGENT_HOST
Ajoute INFRA_006_AGENT_RESOURCE_CHECK.sh, meme principe qu'ES_B001_RAM_CHECK
(ELK_HOST) mais pour VM2/agents : verifie vCPU/RAM/disque AVANT toute
installation, echec dur si sous le seuil. Devient le point d'entree unique
du role AGENT_HOST - FB_001, INFRA_002 et WAG_001 (jusque-la trois entrees
independantes) en dependent desormais tous.

Nouveaux seuils dans vars.conf : MIN_RAM_GB_REQUIRED_AGENT (2 Go),
MIN_DISK_GB_REQUIRED_AGENT (15 Go), MIN_VCPU_REQUIRED_AGENT (1) - bas car
Filebeat/Metricbeat/agent Wazuh sont des binaires legers, sans JVM.

Classeur Excel mis a jour en consequence (feuille "Deploiement VM2") -
l'ancienne note "aucun controle automatique n'existe" est desormais fausse
et a ete corrigee.

Non teste sur une vraie VM2 (jamais deployee a ce jour) - a confirmer au
premier lancement reel, meme discipline honnete que le reste du projet.
</commit_message>
<xml_diff>
--- a/docs/TABLEAU_DE_BORD_EXPLOITATION.xlsx
+++ b/docs/TABLEAU_DE_BORD_EXPLOITATION.xlsx
@@ -2474,7 +2474,7 @@
     <row r="2" ht="32">
       <c r="A2" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">⚠ Rien de ce qui suit dans la section 0 n'est fait par l'orchestrateur - ce sont des prerequis SYSTEME (reseau, ressources), verifies ici a la main une seule fois avant le premier lancement. Aucun controle RAM/disque automatique n'existe pour AGENT_HOST (contrairement a VM1, voir ES_B001_RAM_CHECK) - limite honnete, a verifier soi-meme.</t>
+          <t xml:space="preserve">⚠ Rien de ce qui suit dans la section 0 n'est fait par l'orchestrateur - ce sont des prerequis SYSTEME (reseau), a faire une seule fois avant le premier lancement. Le controle des ressources (RAM/disque/vCPU), lui, EST desormais automatique : voir INFRA_006_AGENT_RESOURCE_CHECK, premier job joue sur AGENT_HOST (bloque tout le reste si la machine est sous le seuil - seuils dans vars.conf : MIN_RAM_GB_REQUIRED_AGENT/MIN_DISK_GB_REQUIRED_AGENT/MIN_VCPU_REQUIRED_AGENT). Ajoute le 2026-08-31, jamais encore teste sur une vraie VM2 - a confirmer au premier lancement reel.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="4">
@@ -2610,7 +2610,7 @@
     <row r="10" ht="18">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7 Verifier les ressources de CETTE machine</t>
+          <t xml:space="preserve">0.7 (Optionnel) Verifier les ressources vous-meme avant de lancer</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="3">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Minimum recommande : 2 vCPU / 4 Go RAM / 20 Go disque (jamais verifie automatiquement pour VM2, a l'inverse de VM1)</t>
+          <t xml:space="preserve">Seuils actuels (vars.conf) : 1 vCPU / 2 Go RAM / 15 Go disque - deja verifie automatiquement par INFRA_006_AGENT_RESOURCE_CHECK au lancement, ceci n'est qu'un controle anticipe</t>
         </is>
       </c>
     </row>

</xml_diff>